<commit_message>
End of Streamlit app
</commit_message>
<xml_diff>
--- a/data/Dengue_Data.xlsx
+++ b/data/Dengue_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MSc-AI\Semester 2\IT5514 -Applied ML\Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dengue_Dashboard\dengue_stats_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81E1A6AF-2665-4F65-9309-B0BBB567F958}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61E36A2A-B869-4589-B1BA-207168ECDAF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545" xr2:uid="{B1BB98B5-0FF4-44C1-B13A-DE7F30100898}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{B1BB98B5-0FF4-44C1-B13A-DE7F30100898}"/>
   </bookViews>
   <sheets>
     <sheet name="WIDE DATA" sheetId="2" r:id="rId1"/>
@@ -154,7 +154,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -175,9 +175,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -215,7 +215,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -321,7 +321,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -463,7 +463,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -471,8 +471,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C85A2C08-8006-4C46-A2CE-82624335577D}">
-  <dimension ref="A1:AB150"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:AB146"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:27">
       <c r="A1" t="s">
@@ -12202,351 +12202,19 @@
       </c>
     </row>
     <row r="142" spans="1:27">
-      <c r="A142" s="1">
-        <v>44440</v>
-      </c>
-      <c r="B142" s="2">
-        <v>0</v>
-      </c>
-      <c r="C142" s="2">
-        <v>0</v>
-      </c>
-      <c r="D142" s="2">
-        <v>0</v>
-      </c>
-      <c r="E142" s="2">
-        <v>0</v>
-      </c>
-      <c r="F142" s="2">
-        <v>0</v>
-      </c>
-      <c r="G142" s="2">
-        <v>0</v>
-      </c>
-      <c r="H142" s="2">
-        <v>0</v>
-      </c>
-      <c r="I142" s="2">
-        <v>0</v>
-      </c>
-      <c r="J142" s="2">
-        <v>0</v>
-      </c>
-      <c r="K142" s="2">
-        <v>0</v>
-      </c>
-      <c r="L142" s="2">
-        <v>0</v>
-      </c>
-      <c r="M142" s="2">
-        <v>0</v>
-      </c>
-      <c r="N142" s="2">
-        <v>0</v>
-      </c>
-      <c r="O142" s="2">
-        <v>0</v>
-      </c>
-      <c r="P142" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q142" s="2">
-        <v>0</v>
-      </c>
-      <c r="R142" s="2">
-        <v>0</v>
-      </c>
-      <c r="S142" s="2">
-        <v>0</v>
-      </c>
-      <c r="T142" s="2">
-        <v>0</v>
-      </c>
-      <c r="U142" s="2">
-        <v>0</v>
-      </c>
-      <c r="V142" s="2">
-        <v>0</v>
-      </c>
-      <c r="W142" s="2">
-        <v>0</v>
-      </c>
-      <c r="X142" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y142" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z142" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA142" s="2">
-        <v>0</v>
-      </c>
+      <c r="A142" s="1"/>
     </row>
     <row r="143" spans="1:27">
-      <c r="A143" s="1">
-        <v>44470</v>
-      </c>
-      <c r="B143" s="2">
-        <v>0</v>
-      </c>
-      <c r="C143" s="2">
-        <v>0</v>
-      </c>
-      <c r="D143" s="2">
-        <v>0</v>
-      </c>
-      <c r="E143" s="2">
-        <v>0</v>
-      </c>
-      <c r="F143" s="2">
-        <v>0</v>
-      </c>
-      <c r="G143" s="2">
-        <v>0</v>
-      </c>
-      <c r="H143" s="2">
-        <v>0</v>
-      </c>
-      <c r="I143" s="2">
-        <v>0</v>
-      </c>
-      <c r="J143" s="2">
-        <v>0</v>
-      </c>
-      <c r="K143" s="2">
-        <v>0</v>
-      </c>
-      <c r="L143" s="2">
-        <v>0</v>
-      </c>
-      <c r="M143" s="2">
-        <v>0</v>
-      </c>
-      <c r="N143" s="2">
-        <v>0</v>
-      </c>
-      <c r="O143" s="2">
-        <v>0</v>
-      </c>
-      <c r="P143" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q143" s="2">
-        <v>0</v>
-      </c>
-      <c r="R143" s="2">
-        <v>0</v>
-      </c>
-      <c r="S143" s="2">
-        <v>0</v>
-      </c>
-      <c r="T143" s="2">
-        <v>0</v>
-      </c>
-      <c r="U143" s="2">
-        <v>0</v>
-      </c>
-      <c r="V143" s="2">
-        <v>0</v>
-      </c>
-      <c r="W143" s="2">
-        <v>0</v>
-      </c>
-      <c r="X143" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y143" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z143" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA143" s="2">
-        <v>0</v>
-      </c>
+      <c r="A143" s="1"/>
     </row>
     <row r="144" spans="1:27">
-      <c r="A144" s="1">
-        <v>44501</v>
-      </c>
-      <c r="B144" s="2">
-        <v>0</v>
-      </c>
-      <c r="C144" s="2">
-        <v>0</v>
-      </c>
-      <c r="D144" s="2">
-        <v>0</v>
-      </c>
-      <c r="E144" s="2">
-        <v>0</v>
-      </c>
-      <c r="F144" s="2">
-        <v>0</v>
-      </c>
-      <c r="G144" s="2">
-        <v>0</v>
-      </c>
-      <c r="H144" s="2">
-        <v>0</v>
-      </c>
-      <c r="I144" s="2">
-        <v>0</v>
-      </c>
-      <c r="J144" s="2">
-        <v>0</v>
-      </c>
-      <c r="K144" s="2">
-        <v>0</v>
-      </c>
-      <c r="L144" s="2">
-        <v>0</v>
-      </c>
-      <c r="M144" s="2">
-        <v>0</v>
-      </c>
-      <c r="N144" s="2">
-        <v>0</v>
-      </c>
-      <c r="O144" s="2">
-        <v>0</v>
-      </c>
-      <c r="P144" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q144" s="2">
-        <v>0</v>
-      </c>
-      <c r="R144" s="2">
-        <v>0</v>
-      </c>
-      <c r="S144" s="2">
-        <v>0</v>
-      </c>
-      <c r="T144" s="2">
-        <v>0</v>
-      </c>
-      <c r="U144" s="2">
-        <v>0</v>
-      </c>
-      <c r="V144" s="2">
-        <v>0</v>
-      </c>
-      <c r="W144" s="2">
-        <v>0</v>
-      </c>
-      <c r="X144" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y144" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z144" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA144" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="145" spans="1:27">
-      <c r="A145" s="1">
-        <v>44531</v>
-      </c>
-      <c r="B145" s="2">
-        <v>0</v>
-      </c>
-      <c r="C145" s="2">
-        <v>0</v>
-      </c>
-      <c r="D145" s="2">
-        <v>0</v>
-      </c>
-      <c r="E145" s="2">
-        <v>0</v>
-      </c>
-      <c r="F145" s="2">
-        <v>0</v>
-      </c>
-      <c r="G145" s="2">
-        <v>0</v>
-      </c>
-      <c r="H145" s="2">
-        <v>0</v>
-      </c>
-      <c r="I145" s="2">
-        <v>0</v>
-      </c>
-      <c r="J145" s="2">
-        <v>0</v>
-      </c>
-      <c r="K145" s="2">
-        <v>0</v>
-      </c>
-      <c r="L145" s="2">
-        <v>0</v>
-      </c>
-      <c r="M145" s="2">
-        <v>0</v>
-      </c>
-      <c r="N145" s="2">
-        <v>0</v>
-      </c>
-      <c r="O145" s="2">
-        <v>0</v>
-      </c>
-      <c r="P145" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q145" s="2">
-        <v>0</v>
-      </c>
-      <c r="R145" s="2">
-        <v>0</v>
-      </c>
-      <c r="S145" s="2">
-        <v>0</v>
-      </c>
-      <c r="T145" s="2">
-        <v>0</v>
-      </c>
-      <c r="U145" s="2">
-        <v>0</v>
-      </c>
-      <c r="V145" s="2">
-        <v>0</v>
-      </c>
-      <c r="W145" s="2">
-        <v>0</v>
-      </c>
-      <c r="X145" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y145" s="2">
-        <v>0</v>
-      </c>
-      <c r="Z145" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA145" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="146" spans="1:27">
+      <c r="A144" s="1"/>
+    </row>
+    <row r="145" spans="1:1">
+      <c r="A145" s="1"/>
+    </row>
+    <row r="146" spans="1:1">
       <c r="A146" s="1"/>
-    </row>
-    <row r="147" spans="1:27">
-      <c r="A147" s="1"/>
-    </row>
-    <row r="148" spans="1:27">
-      <c r="A148" s="1"/>
-    </row>
-    <row r="149" spans="1:27">
-      <c r="A149" s="1"/>
-    </row>
-    <row r="150" spans="1:27">
-      <c r="A150" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12556,7 +12224,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA22ADF2-1046-4FDB-B299-6DEA53AA3411}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">

</xml_diff>